<commit_message>
feat: 重构 daily_quotes 表结构，支持 OHLC 数据
</commit_message>
<xml_diff>
--- a/data/数据库表导出_v3.xlsx
+++ b/data/数据库表导出_v3.xlsx
@@ -614,6 +614,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9.75"/>
+        <color rgb="FF4C4F69"/>
+        <rFont val="Roboto"/>
+        <charset val="134"/>
+      </rPr>
       <t>载体</t>
     </r>
     <r>
@@ -655,6 +661,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9.75"/>
+        <color rgb="FF4C4F69"/>
+        <rFont val="Roboto"/>
+        <charset val="134"/>
+      </rPr>
       <t>操作</t>
     </r>
     <r>
@@ -714,6 +726,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9.75"/>
+        <color rgb="FF4C4F69"/>
+        <rFont val="Roboto"/>
+        <charset val="134"/>
+      </rPr>
       <t>逻辑</t>
     </r>
     <r>
@@ -767,6 +785,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9.75"/>
+        <color rgb="FF4C4F69"/>
+        <rFont val="Roboto"/>
+        <charset val="134"/>
+      </rPr>
       <t>载体</t>
     </r>
     <r>
@@ -808,6 +832,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9.75"/>
+        <color rgb="FF4C4F69"/>
+        <rFont val="Roboto"/>
+        <charset val="134"/>
+      </rPr>
       <t>操作</t>
     </r>
     <r>
@@ -840,6 +870,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9.75"/>
+        <color rgb="FF4C4F69"/>
+        <rFont val="Roboto"/>
+        <charset val="134"/>
+      </rPr>
       <t>逻辑</t>
     </r>
     <r>
@@ -1041,6 +1077,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9.75"/>
+        <color rgb="FF4C4F69"/>
+        <rFont val="Roboto"/>
+        <charset val="134"/>
+      </rPr>
       <t>条 1：</t>
     </r>
     <r>
@@ -1109,6 +1151,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9.75"/>
+        <color rgb="FF4C4F69"/>
+        <rFont val="Roboto"/>
+        <charset val="134"/>
+      </rPr>
       <t>条 2：</t>
     </r>
     <r>
@@ -1177,6 +1225,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9.75"/>
+        <color rgb="FF4C4F69"/>
+        <rFont val="Roboto"/>
+        <charset val="134"/>
+      </rPr>
       <t>条 3：</t>
     </r>
     <r>
@@ -1245,6 +1299,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9.75"/>
+        <color rgb="FF4C4F69"/>
+        <rFont val="Roboto"/>
+        <charset val="134"/>
+      </rPr>
       <t>条 4：</t>
     </r>
     <r>
@@ -1313,6 +1373,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9.75"/>
+        <color rgb="FF4C4F69"/>
+        <rFont val="Roboto"/>
+        <charset val="134"/>
+      </rPr>
       <t>你的系统在生成信号时，只要再加一个条件：</t>
     </r>
     <r>
@@ -2141,7 +2207,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2184,9 +2250,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2609,7 +2672,7 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="31" t="s">
+      <c r="G1" s="30" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
@@ -2635,767 +2698,767 @@
       </c>
     </row>
     <row r="2" spans="1:14">
-      <c r="A2" s="19" t="str">
-        <f>VLOOKUP(B2,$B$24:$C$40,2,0)</f>
+      <c r="A2" s="2" t="str">
+        <f t="shared" ref="A2:A18" si="0">VLOOKUP(B2,$B$24:$C$40,2,0)</f>
         <v>002183</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="19" t="s">
+      <c r="D2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E2" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="F2" s="19" t="s">
+      <c r="E2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="32" t="s">
+      <c r="G2" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="H2" s="19" t="s">
+      <c r="H2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I2" s="19" t="s">
+      <c r="I2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="J2" s="19" t="s">
+      <c r="J2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="K2" s="19" t="s">
+      <c r="K2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="L2" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="M2" s="19" t="s">
+      <c r="L2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N2" s="19" t="s">
+      <c r="N2" s="2" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:14">
-      <c r="A3" s="19" t="str">
-        <f>VLOOKUP(B3,$B$24:$C$40,2,0)</f>
+      <c r="A3" s="2" t="str">
+        <f t="shared" si="0"/>
         <v>005693</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G3" s="32" t="s">
+      <c r="G3" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="H3" s="19" t="s">
+      <c r="H3" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="I3" s="19" t="s">
+      <c r="I3" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="J3" s="19" t="s">
+      <c r="J3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="K3" s="19" t="s">
+      <c r="K3" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="L3" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="M3" s="19" t="s">
+      <c r="L3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M3" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="N3" s="19" t="s">
+      <c r="N3" s="2" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:14">
-      <c r="A4" s="19" t="str">
-        <f>VLOOKUP(B4,$B$24:$C$40,2,0)</f>
+      <c r="A4" s="2" t="str">
+        <f t="shared" si="0"/>
         <v>008702</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="E4" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G4" s="32" t="s">
+      <c r="G4" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="H4" s="19" t="s">
+      <c r="H4" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="I4" s="19" t="s">
+      <c r="I4" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="J4" s="19" t="s">
+      <c r="J4" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="K4" s="19" t="s">
+      <c r="K4" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="L4" s="19" t="s">
+      <c r="L4" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="M4" s="19" t="s">
+      <c r="M4" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="N4" s="19" t="s">
+      <c r="N4" s="2" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:14">
-      <c r="A5" s="19" t="str">
-        <f>VLOOKUP(B5,$B$24:$C$40,2,0)</f>
+      <c r="A5" s="2" t="str">
+        <f t="shared" si="0"/>
         <v>009034</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E5" s="19" t="s">
+      <c r="E5" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="F5" s="19" t="s">
+      <c r="F5" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G5" s="32" t="s">
+      <c r="G5" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="H5" s="19" t="s">
+      <c r="H5" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="I5" s="19" t="s">
+      <c r="I5" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="J5" s="19" t="s">
+      <c r="J5" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="K5" s="19" t="s">
+      <c r="K5" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="L5" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="M5" s="19" t="s">
+      <c r="L5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M5" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="N5" s="19" t="s">
+      <c r="N5" s="2" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:14">
-      <c r="A6" s="19" t="str">
-        <f>VLOOKUP(B6,$B$24:$C$40,2,0)</f>
+      <c r="A6" s="2" t="str">
+        <f t="shared" si="0"/>
         <v>009505</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="E6" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="F6" s="19" t="s">
+      <c r="F6" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G6" s="32" t="s">
+      <c r="G6" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="H6" s="19" t="s">
+      <c r="H6" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="I6" s="19" t="s">
+      <c r="I6" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="J6" s="19" t="s">
+      <c r="J6" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="K6" s="19" t="s">
+      <c r="K6" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="L6" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="M6" s="19" t="s">
+      <c r="L6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M6" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="N6" s="19" t="s">
+      <c r="N6" s="2" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:14">
-      <c r="A7" s="19" t="str">
-        <f>VLOOKUP(B7,$B$24:$C$40,2,0)</f>
+      <c r="A7" s="2" t="str">
+        <f t="shared" si="0"/>
         <v>014662</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G7" s="32" t="s">
+      <c r="G7" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="H7" s="19" t="s">
+      <c r="H7" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="I7" s="19" t="s">
+      <c r="I7" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="J7" s="19" t="s">
+      <c r="J7" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="K7" s="19" t="s">
+      <c r="K7" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="L7" s="19" t="s">
+      <c r="L7" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="M7" s="19" t="s">
+      <c r="M7" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="N7" s="19" t="s">
+      <c r="N7" s="2" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:14">
-      <c r="A8" s="19" t="str">
-        <f>VLOOKUP(B8,$B$24:$C$40,2,0)</f>
+      <c r="A8" s="2" t="str">
+        <f t="shared" si="0"/>
         <v>014881</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="E8" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="F8" s="19" t="s">
+      <c r="F8" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G8" s="32" t="s">
+      <c r="G8" s="31" t="s">
         <v>69</v>
       </c>
-      <c r="H8" s="19" t="s">
+      <c r="H8" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="I8" s="19" t="s">
+      <c r="I8" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="J8" s="19" t="s">
+      <c r="J8" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="K8" s="19" t="s">
+      <c r="K8" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="L8" s="19" t="s">
+      <c r="L8" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="M8" s="19" t="s">
+      <c r="M8" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="N8" s="19" t="s">
+      <c r="N8" s="2" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:14">
-      <c r="A9" s="19" t="str">
-        <f>VLOOKUP(B9,$B$24:$C$40,2,0)</f>
+      <c r="A9" s="2" t="str">
+        <f t="shared" si="0"/>
         <v>017470</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E9" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="F9" s="19" t="s">
+      <c r="F9" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G9" s="32" t="s">
+      <c r="G9" s="31" t="s">
         <v>78</v>
       </c>
-      <c r="H9" s="19" t="s">
+      <c r="H9" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="I9" s="19" t="s">
+      <c r="I9" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="J9" s="19" t="s">
+      <c r="J9" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="K9" s="19" t="s">
+      <c r="K9" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="L9" s="19" t="s">
+      <c r="L9" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="M9" s="19" t="s">
+      <c r="M9" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="N9" s="19" t="s">
+      <c r="N9" s="2" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="10" spans="1:14">
-      <c r="A10" s="19" t="str">
-        <f>VLOOKUP(B10,$B$24:$C$40,2,0)</f>
+      <c r="A10" s="2" t="str">
+        <f t="shared" si="0"/>
         <v>018345</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="19" t="s">
+      <c r="E10" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="F10" s="19" t="s">
+      <c r="F10" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G10" s="32" t="s">
+      <c r="G10" s="31" t="s">
         <v>69</v>
       </c>
-      <c r="H10" s="19" t="s">
+      <c r="H10" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="I10" s="19" t="s">
+      <c r="I10" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="J10" s="19" t="s">
+      <c r="J10" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="K10" s="19" t="s">
+      <c r="K10" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="L10" s="19" t="s">
+      <c r="L10" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="M10" s="19" t="s">
+      <c r="M10" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="N10" s="19" t="s">
+      <c r="N10" s="2" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="11" spans="1:14">
-      <c r="A11" s="19" t="str">
-        <f>VLOOKUP(B11,$B$24:$C$40,2,0)</f>
+      <c r="A11" s="2" t="str">
+        <f t="shared" si="0"/>
         <v>020341</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="D11" s="19" t="s">
+      <c r="D11" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E11" s="19" t="s">
+      <c r="E11" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F11" s="19" t="s">
+      <c r="F11" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G11" s="32" t="s">
+      <c r="G11" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="H11" s="19" t="s">
+      <c r="H11" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="I11" s="19" t="s">
+      <c r="I11" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="J11" s="19" t="s">
+      <c r="J11" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="K11" s="19" t="s">
+      <c r="K11" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="L11" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="M11" s="19" t="s">
+      <c r="L11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M11" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="N11" s="19" t="s">
+      <c r="N11" s="2" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="12" spans="1:14">
-      <c r="A12" s="19" t="str">
-        <f>VLOOKUP(B12,$B$24:$C$40,2,0)</f>
+      <c r="A12" s="2" t="str">
+        <f t="shared" si="0"/>
         <v>020482</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="C12" s="19" t="s">
+      <c r="C12" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D12" s="19" t="s">
+      <c r="D12" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E12" s="19" t="s">
+      <c r="E12" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="F12" s="19" t="s">
+      <c r="F12" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G12" s="32" t="s">
+      <c r="G12" s="31" t="s">
         <v>69</v>
       </c>
-      <c r="H12" s="19" t="s">
+      <c r="H12" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="I12" s="19" t="s">
+      <c r="I12" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="J12" s="19" t="s">
+      <c r="J12" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="K12" s="19" t="s">
+      <c r="K12" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="L12" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="M12" s="19" t="s">
+      <c r="L12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M12" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="N12" s="19" t="s">
+      <c r="N12" s="2" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="13" spans="1:14">
-      <c r="A13" s="19" t="str">
-        <f>VLOOKUP(B13,$B$24:$C$40,2,0)</f>
+      <c r="A13" s="2" t="str">
+        <f t="shared" si="0"/>
         <v>159227</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C13" s="19" t="s">
+      <c r="C13" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D13" s="19" t="s">
+      <c r="D13" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E13" s="19" t="s">
+      <c r="E13" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F13" s="19" t="s">
+      <c r="F13" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G13" s="32" t="s">
+      <c r="G13" s="31" t="s">
         <v>102</v>
       </c>
-      <c r="H13" s="19" t="s">
+      <c r="H13" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="I13" s="19" t="s">
+      <c r="I13" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="J13" s="19" t="s">
+      <c r="J13" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="K13" s="19" t="s">
+      <c r="K13" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="L13" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="M13" s="19" t="s">
+      <c r="L13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M13" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="N13" s="19" t="s">
+      <c r="N13" s="2" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="14" spans="1:14">
-      <c r="A14" s="19" t="str">
-        <f>VLOOKUP(B14,$B$24:$C$40,2,0)</f>
+      <c r="A14" s="2" t="str">
+        <f t="shared" si="0"/>
         <v>159241</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="C14" s="19" t="s">
+      <c r="C14" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D14" s="19" t="s">
+      <c r="D14" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E14" s="19" t="s">
+      <c r="E14" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F14" s="19" t="s">
+      <c r="F14" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G14" s="32" t="s">
+      <c r="G14" s="31" t="s">
         <v>102</v>
       </c>
-      <c r="H14" s="19" t="s">
+      <c r="H14" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="I14" s="19" t="s">
+      <c r="I14" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="J14" s="19" t="s">
+      <c r="J14" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="K14" s="19" t="s">
+      <c r="K14" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="L14" s="19" t="s">
+      <c r="L14" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="M14" s="19" t="s">
+      <c r="M14" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="N14" s="19" t="s">
+      <c r="N14" s="2" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="15" spans="1:14">
-      <c r="A15" s="19" t="str">
-        <f>VLOOKUP(B15,$B$24:$C$40,2,0)</f>
+      <c r="A15" s="2" t="str">
+        <f t="shared" si="0"/>
         <v>159530</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="C15" s="19" t="s">
+      <c r="C15" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="D15" s="19" t="s">
+      <c r="D15" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E15" s="19" t="s">
+      <c r="E15" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="F15" s="19" t="s">
+      <c r="F15" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G15" s="32" t="s">
+      <c r="G15" s="31" t="s">
         <v>69</v>
       </c>
-      <c r="H15" s="19" t="s">
+      <c r="H15" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="I15" s="19" t="s">
+      <c r="I15" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="J15" s="19" t="s">
+      <c r="J15" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="K15" s="19" t="s">
+      <c r="K15" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="L15" s="19" t="s">
+      <c r="L15" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="M15" s="19" t="s">
+      <c r="M15" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="N15" s="19" t="s">
+      <c r="N15" s="2" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="16" spans="1:14">
-      <c r="A16" s="19" t="str">
-        <f>VLOOKUP(B16,$B$24:$C$40,2,0)</f>
+      <c r="A16" s="2" t="str">
+        <f t="shared" si="0"/>
         <v>159770</v>
       </c>
-      <c r="B16" s="19" t="s">
+      <c r="B16" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="C16" s="19" t="s">
+      <c r="C16" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D16" s="19" t="s">
+      <c r="D16" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E16" s="19" t="s">
+      <c r="E16" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="F16" s="19" t="s">
+      <c r="F16" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G16" s="32" t="s">
+      <c r="G16" s="31" t="s">
         <v>69</v>
       </c>
-      <c r="H16" s="19" t="s">
+      <c r="H16" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="I16" s="19" t="s">
+      <c r="I16" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="J16" s="19" t="s">
+      <c r="J16" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="K16" s="19" t="s">
+      <c r="K16" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="L16" s="19" t="s">
+      <c r="L16" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="M16" s="19" t="s">
+      <c r="M16" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="N16" s="19" t="s">
+      <c r="N16" s="2" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="17" spans="1:14">
-      <c r="A17" s="19" t="str">
-        <f>VLOOKUP(B17,$B$24:$C$40,2,0)</f>
+      <c r="A17" s="2" t="str">
+        <f t="shared" si="0"/>
         <v>159781</v>
       </c>
-      <c r="B17" s="19" t="s">
+      <c r="B17" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="C17" s="19" t="s">
+      <c r="C17" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="D17" s="19" t="s">
+      <c r="D17" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E17" s="19" t="s">
+      <c r="E17" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="F17" s="19" t="s">
+      <c r="F17" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G17" s="32" t="s">
+      <c r="G17" s="31" t="s">
         <v>123</v>
       </c>
-      <c r="H17" s="19" t="s">
+      <c r="H17" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="I17" s="19" t="s">
+      <c r="I17" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="J17" s="19" t="s">
+      <c r="J17" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="K17" s="19" t="s">
+      <c r="K17" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="L17" s="19" t="s">
+      <c r="L17" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="M17" s="19" t="s">
+      <c r="M17" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="N17" s="19" t="s">
+      <c r="N17" s="2" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="18" spans="1:14">
-      <c r="A18" s="19" t="str">
-        <f>VLOOKUP(B18,$B$24:$C$40,2,0)</f>
+      <c r="A18" s="2" t="str">
+        <f t="shared" si="0"/>
         <v>159792</v>
       </c>
-      <c r="B18" s="19" t="s">
+      <c r="B18" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="C18" s="19" t="s">
+      <c r="C18" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D18" s="19" t="s">
+      <c r="D18" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E18" s="19" t="s">
+      <c r="E18" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="F18" s="19" t="s">
+      <c r="F18" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G18" s="32" t="s">
+      <c r="G18" s="31" t="s">
         <v>130</v>
       </c>
-      <c r="H18" s="19" t="s">
+      <c r="H18" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="I18" s="19" t="s">
+      <c r="I18" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="J18" s="19" t="s">
+      <c r="J18" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="K18" s="19" t="s">
+      <c r="K18" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="L18" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="M18" s="19" t="s">
+      <c r="L18" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M18" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="N18" s="19" t="s">
+      <c r="N18" s="2" t="s">
         <v>133</v>
       </c>
     </row>
@@ -3496,7 +3559,7 @@
       </c>
     </row>
     <row r="35" spans="2:3">
-      <c r="B35" s="19" t="s">
+      <c r="B35" s="2" t="s">
         <v>99</v>
       </c>
       <c r="C35" s="3" t="s">
@@ -3504,7 +3567,7 @@
       </c>
     </row>
     <row r="36" spans="2:3">
-      <c r="B36" s="19" t="s">
+      <c r="B36" s="2" t="s">
         <v>106</v>
       </c>
       <c r="C36" s="3" t="s">
@@ -3512,7 +3575,7 @@
       </c>
     </row>
     <row r="37" spans="2:3">
-      <c r="B37" s="19" t="s">
+      <c r="B37" s="2" t="s">
         <v>109</v>
       </c>
       <c r="C37" s="3" t="s">
@@ -3520,7 +3583,7 @@
       </c>
     </row>
     <row r="38" spans="2:3">
-      <c r="B38" s="19" t="s">
+      <c r="B38" s="2" t="s">
         <v>116</v>
       </c>
       <c r="C38" s="3" t="s">
@@ -3528,7 +3591,7 @@
       </c>
     </row>
     <row r="39" spans="2:3">
-      <c r="B39" s="19" t="s">
+      <c r="B39" s="2" t="s">
         <v>121</v>
       </c>
       <c r="C39" s="3" t="s">
@@ -3536,7 +3599,7 @@
       </c>
     </row>
     <row r="40" spans="2:3">
-      <c r="B40" s="19" t="s">
+      <c r="B40" s="2" t="s">
         <v>128</v>
       </c>
       <c r="C40" s="3" t="s">
@@ -3645,1146 +3708,1146 @@
       </c>
     </row>
     <row r="2" spans="1:21">
-      <c r="A2" s="19">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" s="20" t="str">
+      <c r="B2" s="19" t="str">
         <f>VLOOKUP(C2,$C$39:$D$55,2,0)</f>
         <v>005693</v>
       </c>
-      <c r="C2" s="20" t="s">
+      <c r="C2" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="19" t="s">
+      <c r="D2" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="E2" s="21">
+      <c r="E2" s="20">
         <v>46088.9471296296</v>
       </c>
-      <c r="F2" s="22">
+      <c r="F2" s="21">
         <v>399.82</v>
       </c>
-      <c r="G2" s="23">
+      <c r="G2" s="22">
         <v>1.4256</v>
       </c>
-      <c r="H2" s="22">
+      <c r="H2" s="21">
         <f t="shared" ref="H2:H17" si="0">F2*0.2</f>
         <v>79.964</v>
       </c>
-      <c r="I2" s="24">
+      <c r="I2" s="23">
         <v>1.4484</v>
       </c>
-      <c r="J2" s="25">
+      <c r="J2" s="24">
         <f t="shared" ref="J2:J17" si="1">I2*F2</f>
         <v>579.099288</v>
       </c>
-      <c r="K2" s="22">
+      <c r="K2" s="21">
         <f t="shared" ref="K2:K17" si="2">F2*G2</f>
         <v>569.983392</v>
       </c>
-      <c r="L2" s="22">
+      <c r="L2" s="21">
         <f t="shared" ref="L2:L17" si="3">J2-K2</f>
         <v>9.11589600000002</v>
       </c>
-      <c r="M2" s="26">
+      <c r="M2" s="25">
         <f t="shared" ref="M2:M17" si="4">L2/K2</f>
         <v>0.015993265993266</v>
       </c>
-      <c r="N2" s="27">
+      <c r="N2" s="26">
         <v>1</v>
       </c>
-      <c r="O2" s="19" t="s">
+      <c r="O2" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="P2" s="19">
+      <c r="P2" s="2">
         <v>100</v>
       </c>
-      <c r="Q2" s="19" t="s">
+      <c r="Q2" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="R2" s="19">
+      <c r="R2" s="2">
         <v>270</v>
       </c>
-      <c r="S2" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="T2" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="U2" s="19" t="s">
+      <c r="S2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U2" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:21">
-      <c r="A3" s="19">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="19" t="str">
+      <c r="B3" s="2" t="str">
         <f t="shared" ref="B3:B11" si="5">VLOOKUP(C3,$C$39:$D$55,2,0)</f>
         <v>008702</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="E3" s="21">
+      <c r="E3" s="20">
         <v>46088.9471296296</v>
       </c>
-      <c r="F3" s="22">
+      <c r="F3" s="21">
         <v>479.56</v>
       </c>
-      <c r="G3" s="23">
+      <c r="G3" s="22">
         <v>2.5023</v>
       </c>
-      <c r="H3" s="22">
+      <c r="H3" s="21">
         <f t="shared" si="0"/>
         <v>95.912</v>
       </c>
-      <c r="I3" s="24">
+      <c r="I3" s="23">
         <v>2.4685</v>
       </c>
-      <c r="J3" s="25">
+      <c r="J3" s="24">
         <f t="shared" si="1"/>
         <v>1183.79386</v>
       </c>
-      <c r="K3" s="22">
+      <c r="K3" s="21">
         <f t="shared" si="2"/>
         <v>1200.002988</v>
       </c>
-      <c r="L3" s="22">
+      <c r="L3" s="21">
         <f t="shared" si="3"/>
         <v>-16.209128</v>
       </c>
-      <c r="M3" s="26">
+      <c r="M3" s="25">
         <f t="shared" si="4"/>
         <v>-0.0135075730328098</v>
       </c>
-      <c r="N3" s="27">
+      <c r="N3" s="26">
         <v>1</v>
       </c>
-      <c r="O3" s="19" t="s">
+      <c r="O3" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="P3" s="19">
+      <c r="P3" s="2">
         <v>200</v>
       </c>
-      <c r="Q3" s="19" t="s">
+      <c r="Q3" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="R3" s="19">
+      <c r="R3" s="2">
         <v>2000</v>
       </c>
-      <c r="S3" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="T3" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="U3" s="19" t="s">
+      <c r="S3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="T3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U3" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:21">
-      <c r="A4" s="19">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="B4" s="19" t="str">
+      <c r="B4" s="2" t="str">
         <f t="shared" si="5"/>
         <v>009034</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="E4" s="21">
+      <c r="E4" s="20">
         <v>46088.9471296296</v>
       </c>
-      <c r="F4" s="22">
+      <c r="F4" s="21">
         <v>383.5</v>
       </c>
-      <c r="G4" s="23">
+      <c r="G4" s="22">
         <v>2.556</v>
       </c>
-      <c r="H4" s="22">
+      <c r="H4" s="21">
         <f t="shared" si="0"/>
         <v>76.7</v>
       </c>
-      <c r="I4" s="24">
+      <c r="I4" s="23">
         <v>2.636</v>
       </c>
-      <c r="J4" s="25">
+      <c r="J4" s="24">
         <f t="shared" si="1"/>
         <v>1010.906</v>
       </c>
-      <c r="K4" s="22">
+      <c r="K4" s="21">
         <f t="shared" si="2"/>
         <v>980.226</v>
       </c>
-      <c r="L4" s="22">
+      <c r="L4" s="21">
         <f t="shared" si="3"/>
         <v>30.6800000000001</v>
       </c>
-      <c r="M4" s="26">
+      <c r="M4" s="25">
         <f t="shared" si="4"/>
         <v>0.0312989045383412</v>
       </c>
-      <c r="N4" s="27">
+      <c r="N4" s="26">
         <v>1</v>
       </c>
-      <c r="O4" s="19" t="s">
+      <c r="O4" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="P4" s="19">
+      <c r="P4" s="2">
         <v>200</v>
       </c>
-      <c r="Q4" s="19" t="s">
+      <c r="Q4" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="R4" s="19">
+      <c r="R4" s="2">
         <v>2200</v>
       </c>
-      <c r="S4" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="T4" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="U4" s="19" t="s">
+      <c r="S4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="T4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U4" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:21">
-      <c r="A5" s="19">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="B5" s="19" t="str">
+      <c r="B5" s="2" t="str">
         <f t="shared" si="5"/>
         <v>009505</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="E5" s="21">
+      <c r="E5" s="20">
         <v>46088.9471296296</v>
       </c>
-      <c r="F5" s="22">
+      <c r="F5" s="21">
         <v>416.65</v>
       </c>
-      <c r="G5" s="23">
+      <c r="G5" s="22">
         <v>2.4001</v>
       </c>
-      <c r="H5" s="22">
+      <c r="H5" s="21">
         <f t="shared" si="0"/>
         <v>83.33</v>
       </c>
-      <c r="I5" s="24">
+      <c r="I5" s="23">
         <v>2.3958</v>
       </c>
-      <c r="J5" s="25">
+      <c r="J5" s="24">
         <f t="shared" si="1"/>
         <v>998.21007</v>
       </c>
-      <c r="K5" s="22">
+      <c r="K5" s="21">
         <f t="shared" si="2"/>
         <v>1000.001665</v>
       </c>
-      <c r="L5" s="22">
+      <c r="L5" s="21">
         <f t="shared" si="3"/>
         <v>-1.79159500000014</v>
       </c>
-      <c r="M5" s="26">
+      <c r="M5" s="25">
         <f t="shared" si="4"/>
         <v>-0.00179159201699943</v>
       </c>
-      <c r="N5" s="27">
+      <c r="N5" s="26">
         <v>1</v>
       </c>
-      <c r="O5" s="19" t="s">
+      <c r="O5" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="P5" s="19">
+      <c r="P5" s="2">
         <v>200</v>
       </c>
-      <c r="Q5" s="19" t="s">
+      <c r="Q5" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="R5" s="19">
+      <c r="R5" s="2">
         <v>2800</v>
       </c>
-      <c r="S5" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="T5" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="U5" s="19" t="s">
+      <c r="S5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="T5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U5" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:21">
-      <c r="A6" s="19">
+      <c r="A6" s="2">
         <v>5</v>
       </c>
-      <c r="B6" s="19" t="str">
+      <c r="B6" s="2" t="str">
         <f t="shared" si="5"/>
         <v>014662</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="E6" s="21">
+      <c r="E6" s="20">
         <v>46088.9471296296</v>
       </c>
-      <c r="F6" s="22">
+      <c r="F6" s="21">
         <v>233.16</v>
       </c>
-      <c r="G6" s="23">
+      <c r="G6" s="22">
         <v>2.5733</v>
       </c>
-      <c r="H6" s="22">
+      <c r="H6" s="21">
         <f t="shared" si="0"/>
         <v>46.632</v>
       </c>
-      <c r="I6" s="24">
+      <c r="I6" s="23">
         <v>2.5423</v>
       </c>
-      <c r="J6" s="25">
+      <c r="J6" s="24">
         <f t="shared" si="1"/>
         <v>592.762668</v>
       </c>
-      <c r="K6" s="22">
+      <c r="K6" s="21">
         <f t="shared" si="2"/>
         <v>599.990628</v>
       </c>
-      <c r="L6" s="22">
+      <c r="L6" s="21">
         <f t="shared" si="3"/>
         <v>-7.22796000000005</v>
       </c>
-      <c r="M6" s="26">
+      <c r="M6" s="25">
         <f t="shared" si="4"/>
         <v>-0.0120467881708313</v>
       </c>
-      <c r="N6" s="27">
+      <c r="N6" s="26">
         <v>1</v>
       </c>
-      <c r="O6" s="19" t="s">
+      <c r="O6" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="P6" s="19">
+      <c r="P6" s="2">
         <v>200</v>
       </c>
-      <c r="Q6" s="19" t="s">
+      <c r="Q6" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="R6" s="19">
+      <c r="R6" s="2">
         <v>5500</v>
       </c>
-      <c r="S6" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="T6" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="U6" s="19" t="s">
+      <c r="S6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="T6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U6" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:21">
-      <c r="A7" s="19">
+      <c r="A7" s="2">
         <v>6</v>
       </c>
-      <c r="B7" s="20" t="str">
+      <c r="B7" s="19" t="str">
         <f t="shared" si="5"/>
         <v>014881</v>
       </c>
-      <c r="C7" s="20" t="s">
+      <c r="C7" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="E7" s="21">
+      <c r="E7" s="20">
         <v>46088.9471296296</v>
       </c>
-      <c r="F7" s="22">
+      <c r="F7" s="21">
         <v>1572.57</v>
       </c>
-      <c r="G7" s="23">
+      <c r="G7" s="22">
         <v>1.2718</v>
       </c>
-      <c r="H7" s="22">
+      <c r="H7" s="21">
         <f t="shared" si="0"/>
         <v>314.514</v>
       </c>
-      <c r="I7" s="24">
+      <c r="I7" s="23">
         <v>1.2077</v>
       </c>
-      <c r="J7" s="25">
+      <c r="J7" s="24">
         <f t="shared" si="1"/>
         <v>1899.192789</v>
       </c>
-      <c r="K7" s="22">
+      <c r="K7" s="21">
         <f t="shared" si="2"/>
         <v>1999.994526</v>
       </c>
-      <c r="L7" s="22">
+      <c r="L7" s="21">
         <f t="shared" si="3"/>
         <v>-100.801737</v>
       </c>
-      <c r="M7" s="26">
+      <c r="M7" s="25">
         <f t="shared" si="4"/>
         <v>-0.0504010064475547</v>
       </c>
-      <c r="N7" s="27">
+      <c r="N7" s="26">
         <v>0</v>
       </c>
-      <c r="O7" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="P7" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q7" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="R7" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="S7" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="T7" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="U7" s="19" t="s">
+      <c r="O7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="P7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="R7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="S7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="T7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U7" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:21">
-      <c r="A8" s="19">
+      <c r="A8" s="2">
         <v>7</v>
       </c>
-      <c r="B8" s="20" t="str">
+      <c r="B8" s="19" t="str">
         <f t="shared" si="5"/>
         <v>017470</v>
       </c>
-      <c r="C8" s="20" t="s">
+      <c r="C8" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="E8" s="21">
+      <c r="E8" s="20">
         <v>46088.9471296296</v>
       </c>
-      <c r="F8" s="22">
+      <c r="F8" s="21">
         <v>433.92</v>
       </c>
-      <c r="G8" s="23">
+      <c r="G8" s="22">
         <v>2.1663</v>
       </c>
-      <c r="H8" s="22">
+      <c r="H8" s="21">
         <f t="shared" si="0"/>
         <v>86.784</v>
       </c>
-      <c r="I8" s="24">
+      <c r="I8" s="23">
         <v>2.1024</v>
       </c>
-      <c r="J8" s="25">
+      <c r="J8" s="24">
         <f t="shared" si="1"/>
         <v>912.273408</v>
       </c>
-      <c r="K8" s="22">
+      <c r="K8" s="21">
         <f t="shared" si="2"/>
         <v>940.000896</v>
       </c>
-      <c r="L8" s="22">
+      <c r="L8" s="21">
         <f t="shared" si="3"/>
         <v>-27.7274880000002</v>
       </c>
-      <c r="M8" s="26">
+      <c r="M8" s="25">
         <f t="shared" si="4"/>
         <v>-0.0294972995429998</v>
       </c>
-      <c r="N8" s="27">
+      <c r="N8" s="26">
         <v>1</v>
       </c>
-      <c r="O8" s="19" t="s">
+      <c r="O8" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="P8" s="19">
+      <c r="P8" s="2">
         <v>100</v>
       </c>
-      <c r="Q8" s="19" t="s">
+      <c r="Q8" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="R8" s="19">
+      <c r="R8" s="2">
         <v>840</v>
       </c>
-      <c r="S8" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="T8" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="U8" s="19" t="s">
+      <c r="S8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="T8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U8" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:21">
-      <c r="A9" s="19">
+      <c r="A9" s="2">
         <v>8</v>
       </c>
-      <c r="B9" s="20" t="str">
+      <c r="B9" s="19" t="str">
         <f t="shared" si="5"/>
         <v>018345</v>
       </c>
-      <c r="C9" s="20" t="s">
+      <c r="C9" s="19" t="s">
         <v>83</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="E9" s="21">
+      <c r="E9" s="20">
         <v>46088.9471296296</v>
       </c>
-      <c r="F9" s="22">
+      <c r="F9" s="21">
         <v>1545.12</v>
       </c>
-      <c r="G9" s="23">
+      <c r="G9" s="22">
         <v>1.2944</v>
       </c>
-      <c r="H9" s="22">
+      <c r="H9" s="21">
         <f t="shared" si="0"/>
         <v>309.024</v>
       </c>
-      <c r="I9" s="24">
+      <c r="I9" s="23">
         <v>1.2294</v>
       </c>
-      <c r="J9" s="25">
+      <c r="J9" s="24">
         <f t="shared" si="1"/>
         <v>1899.570528</v>
       </c>
-      <c r="K9" s="22">
+      <c r="K9" s="21">
         <f t="shared" si="2"/>
         <v>2000.003328</v>
       </c>
-      <c r="L9" s="22">
+      <c r="L9" s="21">
         <f t="shared" si="3"/>
         <v>-100.4328</v>
       </c>
-      <c r="M9" s="26">
+      <c r="M9" s="25">
         <f t="shared" si="4"/>
         <v>-0.0502163164400494</v>
       </c>
-      <c r="N9" s="27">
+      <c r="N9" s="26">
         <v>0</v>
       </c>
-      <c r="O9" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="P9" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q9" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="R9" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="S9" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="T9" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="U9" s="19" t="s">
+      <c r="O9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="P9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="R9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="S9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="T9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U9" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:21">
-      <c r="A10" s="19">
+      <c r="A10" s="2">
         <v>9</v>
       </c>
-      <c r="B10" s="19" t="str">
+      <c r="B10" s="2" t="str">
         <f t="shared" si="5"/>
         <v>020341</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="E10" s="21">
+      <c r="E10" s="20">
         <v>46088.9471296296</v>
       </c>
-      <c r="F10" s="22">
+      <c r="F10" s="21">
         <v>388.55</v>
       </c>
-      <c r="G10" s="23">
+      <c r="G10" s="22">
         <v>2.5737</v>
       </c>
-      <c r="H10" s="22">
+      <c r="H10" s="21">
         <f t="shared" si="0"/>
         <v>77.71</v>
       </c>
-      <c r="I10" s="24">
+      <c r="I10" s="23">
         <v>2.5857</v>
       </c>
-      <c r="J10" s="25">
+      <c r="J10" s="24">
         <f t="shared" si="1"/>
         <v>1004.673735</v>
       </c>
-      <c r="K10" s="22">
+      <c r="K10" s="21">
         <f t="shared" si="2"/>
         <v>1000.011135</v>
       </c>
-      <c r="L10" s="22">
+      <c r="L10" s="21">
         <f t="shared" si="3"/>
         <v>4.6626</v>
       </c>
-      <c r="M10" s="26">
+      <c r="M10" s="25">
         <f t="shared" si="4"/>
         <v>0.0046625480825271</v>
       </c>
-      <c r="N10" s="27">
+      <c r="N10" s="26">
         <v>1</v>
       </c>
-      <c r="O10" s="19" t="s">
+      <c r="O10" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="P10" s="19">
+      <c r="P10" s="2">
         <v>200</v>
       </c>
-      <c r="Q10" s="19" t="s">
+      <c r="Q10" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="R10" s="19">
+      <c r="R10" s="2">
         <v>2000</v>
       </c>
-      <c r="S10" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="T10" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="U10" s="19" t="s">
+      <c r="S10" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="T10" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U10" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:21">
-      <c r="A11" s="19">
+      <c r="A11" s="2">
         <v>10</v>
       </c>
-      <c r="B11" s="20" t="str">
+      <c r="B11" s="19" t="str">
         <f t="shared" si="5"/>
         <v>020482</v>
       </c>
-      <c r="C11" s="20" t="s">
+      <c r="C11" s="19" t="s">
         <v>93</v>
       </c>
-      <c r="D11" s="19" t="s">
+      <c r="D11" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="E11" s="21">
+      <c r="E11" s="20">
         <v>46088.9471296296</v>
       </c>
-      <c r="F11" s="22">
+      <c r="F11" s="21">
         <v>1209.85</v>
       </c>
-      <c r="G11" s="23">
+      <c r="G11" s="22">
         <v>1.6531</v>
       </c>
-      <c r="H11" s="22">
+      <c r="H11" s="21">
         <f t="shared" si="0"/>
         <v>241.97</v>
       </c>
-      <c r="I11" s="24">
+      <c r="I11" s="23">
         <v>1.57</v>
       </c>
-      <c r="J11" s="25">
+      <c r="J11" s="24">
         <f t="shared" si="1"/>
         <v>1899.4645</v>
       </c>
-      <c r="K11" s="22">
+      <c r="K11" s="21">
         <f t="shared" si="2"/>
         <v>2000.003035</v>
       </c>
-      <c r="L11" s="22">
+      <c r="L11" s="21">
         <f t="shared" si="3"/>
         <v>-100.538535</v>
       </c>
-      <c r="M11" s="26">
+      <c r="M11" s="25">
         <f t="shared" si="4"/>
         <v>-0.0502691912165023</v>
       </c>
-      <c r="N11" s="27">
+      <c r="N11" s="26">
         <v>0</v>
       </c>
-      <c r="O11" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="P11" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q11" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="R11" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="S11" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="T11" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="U11" s="19" t="s">
+      <c r="O11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="P11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="R11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="S11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="T11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U11" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:21">
-      <c r="A12" s="19">
+      <c r="A12" s="2">
         <v>11</v>
       </c>
-      <c r="B12" s="33" t="s">
+      <c r="B12" s="32" t="s">
         <v>145</v>
       </c>
-      <c r="C12" s="20" t="s">
+      <c r="C12" s="19" t="s">
         <v>99</v>
       </c>
-      <c r="D12" s="19" t="s">
+      <c r="D12" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="E12" s="21">
+      <c r="E12" s="20">
         <v>46088.9471296296</v>
       </c>
-      <c r="F12" s="22">
+      <c r="F12" s="21">
         <v>600</v>
       </c>
-      <c r="G12" s="23">
+      <c r="G12" s="22">
         <v>1.506</v>
       </c>
-      <c r="H12" s="22">
+      <c r="H12" s="21">
         <f t="shared" si="0"/>
         <v>120</v>
       </c>
-      <c r="I12" s="24">
+      <c r="I12" s="23">
         <v>1.498</v>
       </c>
-      <c r="J12" s="25">
+      <c r="J12" s="24">
         <f t="shared" si="1"/>
         <v>898.8</v>
       </c>
-      <c r="K12" s="22">
+      <c r="K12" s="21">
         <f t="shared" si="2"/>
         <v>903.6</v>
       </c>
-      <c r="L12" s="22">
+      <c r="L12" s="21">
         <f t="shared" si="3"/>
         <v>-4.80000000000007</v>
       </c>
-      <c r="M12" s="26">
+      <c r="M12" s="25">
         <f t="shared" si="4"/>
         <v>-0.00531208499335997</v>
       </c>
-      <c r="N12" s="27">
+      <c r="N12" s="26">
         <v>0</v>
       </c>
-      <c r="O12" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="P12" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q12" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="R12" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="S12" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="T12" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="U12" s="19" t="s">
+      <c r="O12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="P12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="R12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="S12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="T12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U12" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:21">
-      <c r="A13" s="19">
+      <c r="A13" s="2">
         <v>12</v>
       </c>
-      <c r="B13" s="33" t="s">
+      <c r="B13" s="32" t="s">
         <v>146</v>
       </c>
-      <c r="C13" s="20" t="s">
+      <c r="C13" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="D13" s="19" t="s">
+      <c r="D13" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="E13" s="21">
+      <c r="E13" s="20">
         <v>46088.9471296296</v>
       </c>
-      <c r="F13" s="22">
+      <c r="F13" s="21">
         <v>600</v>
       </c>
-      <c r="G13" s="23">
+      <c r="G13" s="22">
         <v>1.538</v>
       </c>
-      <c r="H13" s="22">
+      <c r="H13" s="21">
         <f t="shared" si="0"/>
         <v>120</v>
       </c>
-      <c r="I13" s="24">
+      <c r="I13" s="23">
         <v>1.528</v>
       </c>
-      <c r="J13" s="25">
+      <c r="J13" s="24">
         <f t="shared" si="1"/>
         <v>916.8</v>
       </c>
-      <c r="K13" s="22">
+      <c r="K13" s="21">
         <f t="shared" si="2"/>
         <v>922.8</v>
       </c>
-      <c r="L13" s="22">
+      <c r="L13" s="21">
         <f t="shared" si="3"/>
         <v>-6</v>
       </c>
-      <c r="M13" s="26">
+      <c r="M13" s="25">
         <f t="shared" si="4"/>
         <v>-0.00650195058517555</v>
       </c>
-      <c r="N13" s="27">
+      <c r="N13" s="26">
         <v>0</v>
       </c>
-      <c r="O13" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="P13" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q13" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="R13" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="S13" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="T13" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="U13" s="19" t="s">
+      <c r="O13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="P13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="R13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="S13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="T13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U13" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:21">
-      <c r="A14" s="19">
+      <c r="A14" s="2">
         <v>13</v>
       </c>
-      <c r="B14" s="33" t="s">
+      <c r="B14" s="32" t="s">
         <v>147</v>
       </c>
-      <c r="C14" s="20" t="s">
+      <c r="C14" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="D14" s="19" t="s">
+      <c r="D14" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="E14" s="21">
+      <c r="E14" s="20">
         <v>46088.9471296296</v>
       </c>
-      <c r="F14" s="22">
+      <c r="F14" s="21">
         <v>1500</v>
       </c>
-      <c r="G14" s="23">
+      <c r="G14" s="22">
         <v>1.609</v>
       </c>
-      <c r="H14" s="22">
+      <c r="H14" s="21">
         <f t="shared" si="0"/>
         <v>300</v>
       </c>
-      <c r="I14" s="24">
+      <c r="I14" s="23">
         <v>1.48</v>
       </c>
-      <c r="J14" s="25">
+      <c r="J14" s="24">
         <f t="shared" si="1"/>
         <v>2220</v>
       </c>
-      <c r="K14" s="22">
+      <c r="K14" s="21">
         <f t="shared" si="2"/>
         <v>2413.5</v>
       </c>
-      <c r="L14" s="22">
+      <c r="L14" s="21">
         <f t="shared" si="3"/>
         <v>-193.5</v>
       </c>
-      <c r="M14" s="26">
+      <c r="M14" s="25">
         <f t="shared" si="4"/>
         <v>-0.0801740211311373</v>
       </c>
-      <c r="N14" s="27">
+      <c r="N14" s="26">
         <v>0</v>
       </c>
-      <c r="O14" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="P14" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q14" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="R14" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="S14" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="T14" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="U14" s="19" t="s">
+      <c r="O14" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="P14" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q14" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="R14" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="S14" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="T14" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U14" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="15" spans="1:21">
-      <c r="A15" s="19">
+      <c r="A15" s="2">
         <v>14</v>
       </c>
-      <c r="B15" s="33" t="s">
+      <c r="B15" s="32" t="s">
         <v>148</v>
       </c>
-      <c r="C15" s="20" t="s">
+      <c r="C15" s="19" t="s">
         <v>116</v>
       </c>
-      <c r="D15" s="19" t="s">
+      <c r="D15" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="E15" s="21">
+      <c r="E15" s="20">
         <v>46088.9471296296</v>
       </c>
-      <c r="F15" s="22">
+      <c r="F15" s="21">
         <v>1600</v>
       </c>
-      <c r="G15" s="23">
+      <c r="G15" s="22">
         <v>1.123</v>
       </c>
-      <c r="H15" s="22">
+      <c r="H15" s="21">
         <f t="shared" si="0"/>
         <v>320</v>
       </c>
-      <c r="I15" s="24">
+      <c r="I15" s="23">
         <v>1.061</v>
       </c>
-      <c r="J15" s="25">
+      <c r="J15" s="24">
         <f t="shared" si="1"/>
         <v>1697.6</v>
       </c>
-      <c r="K15" s="22">
+      <c r="K15" s="21">
         <f t="shared" si="2"/>
         <v>1796.8</v>
       </c>
-      <c r="L15" s="22">
+      <c r="L15" s="21">
         <f t="shared" si="3"/>
         <v>-99.2</v>
       </c>
-      <c r="M15" s="26">
+      <c r="M15" s="25">
         <f t="shared" si="4"/>
         <v>-0.0552092609082814</v>
       </c>
-      <c r="N15" s="27">
+      <c r="N15" s="26">
         <v>0</v>
       </c>
-      <c r="O15" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="P15" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q15" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="R15" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="S15" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="T15" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="U15" s="19" t="s">
+      <c r="O15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="P15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="R15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="S15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="T15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U15" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:21">
-      <c r="A16" s="19">
+      <c r="A16" s="2">
         <v>15</v>
       </c>
-      <c r="B16" s="33" t="s">
+      <c r="B16" s="32" t="s">
         <v>149</v>
       </c>
-      <c r="C16" s="20" t="s">
+      <c r="C16" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="D16" s="19" t="s">
+      <c r="D16" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="E16" s="21">
+      <c r="E16" s="20">
         <v>46088.9471296296</v>
       </c>
-      <c r="F16" s="22">
+      <c r="F16" s="21">
         <v>1500</v>
       </c>
-      <c r="G16" s="23">
+      <c r="G16" s="22">
         <v>0.938</v>
       </c>
-      <c r="H16" s="22">
+      <c r="H16" s="21">
         <f t="shared" si="0"/>
         <v>300</v>
       </c>
-      <c r="I16" s="24">
+      <c r="I16" s="23">
         <v>0.92</v>
       </c>
-      <c r="J16" s="25">
+      <c r="J16" s="24">
         <f t="shared" si="1"/>
         <v>1380</v>
       </c>
-      <c r="K16" s="22">
+      <c r="K16" s="21">
         <f t="shared" si="2"/>
         <v>1407</v>
       </c>
-      <c r="L16" s="22">
+      <c r="L16" s="21">
         <f t="shared" si="3"/>
         <v>-27</v>
       </c>
-      <c r="M16" s="26">
+      <c r="M16" s="25">
         <f t="shared" si="4"/>
         <v>-0.0191897654584222</v>
       </c>
-      <c r="N16" s="27">
+      <c r="N16" s="26">
         <v>0</v>
       </c>
-      <c r="O16" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="P16" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q16" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="R16" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="S16" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="T16" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="U16" s="19" t="s">
+      <c r="O16" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="P16" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q16" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="R16" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="S16" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="T16" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U16" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:21">
-      <c r="A17" s="19">
+      <c r="A17" s="2">
         <v>16</v>
       </c>
-      <c r="B17" s="33" t="s">
+      <c r="B17" s="32" t="s">
         <v>150</v>
       </c>
-      <c r="C17" s="20" t="s">
+      <c r="C17" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="D17" s="19" t="s">
+      <c r="D17" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="E17" s="21">
+      <c r="E17" s="20">
         <v>46088.9471296296</v>
       </c>
-      <c r="F17" s="22">
+      <c r="F17" s="21">
         <v>200</v>
       </c>
-      <c r="G17" s="23">
+      <c r="G17" s="22">
         <v>0.786</v>
       </c>
-      <c r="H17" s="22">
+      <c r="H17" s="21">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="I17" s="24">
+      <c r="I17" s="23">
         <v>0.737</v>
       </c>
-      <c r="J17" s="25">
+      <c r="J17" s="24">
         <f t="shared" si="1"/>
         <v>147.4</v>
       </c>
-      <c r="K17" s="22">
+      <c r="K17" s="21">
         <f t="shared" si="2"/>
         <v>157.2</v>
       </c>
-      <c r="L17" s="22">
+      <c r="L17" s="21">
         <f t="shared" si="3"/>
         <v>-9.80000000000001</v>
       </c>
-      <c r="M17" s="26">
+      <c r="M17" s="25">
         <f t="shared" si="4"/>
         <v>-0.0623409669211197</v>
       </c>
-      <c r="N17" s="27">
+      <c r="N17" s="26">
         <v>0</v>
       </c>
-      <c r="O17" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="P17" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q17" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="R17" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="S17" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="T17" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="U17" s="19" t="s">
+      <c r="O17" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="P17" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q17" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="R17" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="S17" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="T17" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U17" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:21">
-      <c r="A18" s="19">
+      <c r="A18" s="2">
         <v>17</v>
       </c>
       <c r="C18" t="s">
         <v>179</v>
       </c>
-      <c r="D18" s="19" t="s">
+      <c r="D18" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="E18" s="21">
+      <c r="E18" s="20">
         <v>46088.9471296296</v>
       </c>
       <c r="J18" s="11">
@@ -4796,71 +4859,71 @@
     </row>
     <row r="19" spans="1:21">
       <c r="A19" s="1"/>
-      <c r="B19" s="19" t="str">
+      <c r="B19" s="2" t="str">
         <f>VLOOKUP(C19,$C$39:$D$55,2,0)</f>
         <v>002183</v>
       </c>
-      <c r="C19" s="19" t="s">
+      <c r="C19" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D19" s="19" t="s">
+      <c r="D19" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="E19" s="21">
+      <c r="E19" s="20">
         <v>46088.9471296296</v>
       </c>
-      <c r="F19" s="22"/>
-      <c r="G19" s="23"/>
-      <c r="H19" s="22"/>
-      <c r="I19" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="J19" s="25">
+      <c r="F19" s="21"/>
+      <c r="G19" s="22"/>
+      <c r="H19" s="21"/>
+      <c r="I19" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="J19" s="24">
         <v>81070.62</v>
       </c>
-      <c r="K19" s="22">
+      <c r="K19" s="21">
         <f>J19</f>
         <v>81070.62</v>
       </c>
-      <c r="L19" s="22">
+      <c r="L19" s="21">
         <v>1064.62</v>
       </c>
-      <c r="M19" s="26">
+      <c r="M19" s="25">
         <f>L19/K19</f>
         <v>0.0131320076249571</v>
       </c>
-      <c r="N19" s="27">
+      <c r="N19" s="26">
         <v>0</v>
       </c>
-      <c r="O19" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="P19" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q19" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="R19" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="S19" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="T19" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="U19" s="19" t="s">
+      <c r="O19" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="P19" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q19" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="R19" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="S19" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="T19" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U19" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="21" spans="1:21">
-      <c r="C21" s="28" t="s">
+      <c r="C21" s="27" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="22" spans="1:21">
-      <c r="C22" s="29"/>
+      <c r="C22" s="28"/>
       <c r="J22" s="11">
         <f>SUM(J2:J17)</f>
         <v>19240.546846</v>
@@ -4873,26 +4936,26 @@
         <f>SUM(L2:L17)</f>
         <v>-650.570747</v>
       </c>
-      <c r="M22" s="30">
+      <c r="M22" s="29">
         <f>L22/K22</f>
         <v>-0.0327065959948347</v>
       </c>
     </row>
     <row r="23" spans="1:21">
-      <c r="C23" s="28" t="s">
+      <c r="C23" s="27" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="24" spans="1:21">
-      <c r="C24" s="29"/>
+      <c r="C24" s="28"/>
     </row>
     <row r="25" spans="1:21">
-      <c r="C25" s="28" t="s">
+      <c r="C25" s="27" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="26" spans="1:21">
-      <c r="C26" s="29"/>
+      <c r="C26" s="28"/>
     </row>
     <row r="27" spans="1:21">
       <c r="C27" s="5" t="s">
@@ -4910,15 +4973,15 @@
       </c>
     </row>
     <row r="30" spans="1:21">
-      <c r="C30" s="29"/>
+      <c r="C30" s="28"/>
     </row>
     <row r="31" spans="1:21">
-      <c r="C31" s="28" t="s">
+      <c r="C31" s="27" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="32" spans="1:21">
-      <c r="C32" s="29"/>
+      <c r="C32" s="28"/>
     </row>
     <row r="33" spans="3:4">
       <c r="C33" s="5" t="s">
@@ -5032,7 +5095,7 @@
       </c>
     </row>
     <row r="50" spans="3:4">
-      <c r="C50" s="19" t="s">
+      <c r="C50" s="2" t="s">
         <v>99</v>
       </c>
       <c r="D50" s="3" t="s">
@@ -5040,7 +5103,7 @@
       </c>
     </row>
     <row r="51" spans="3:4">
-      <c r="C51" s="19" t="s">
+      <c r="C51" s="2" t="s">
         <v>106</v>
       </c>
       <c r="D51" s="3" t="s">
@@ -5048,7 +5111,7 @@
       </c>
     </row>
     <row r="52" spans="3:4">
-      <c r="C52" s="19" t="s">
+      <c r="C52" s="2" t="s">
         <v>109</v>
       </c>
       <c r="D52" s="3" t="s">
@@ -5056,7 +5119,7 @@
       </c>
     </row>
     <row r="53" spans="3:4">
-      <c r="C53" s="19" t="s">
+      <c r="C53" s="2" t="s">
         <v>116</v>
       </c>
       <c r="D53" s="3" t="s">
@@ -5064,7 +5127,7 @@
       </c>
     </row>
     <row r="54" spans="3:4">
-      <c r="C54" s="19" t="s">
+      <c r="C54" s="2" t="s">
         <v>121</v>
       </c>
       <c r="D54" s="3" t="s">
@@ -5072,7 +5135,7 @@
       </c>
     </row>
     <row r="55" spans="3:4">
-      <c r="C55" s="19" t="s">
+      <c r="C55" s="2" t="s">
         <v>128</v>
       </c>
       <c r="D55" s="3" t="s">

</xml_diff>